<commit_message>
Changement fichiers et script d'intégration des métadonnées et script de création de la base : 1) ajout des métadonnées de localisation dans le fichier des instruments et ajout des groupes dans le fichier des personnes 2) Dans integration_metadonnees.py : ajout des requêtes pour intégrer les groupes et les projet + correction des requêtes comportant ON CONFLICT ... DO NOTHING par WHERE NOT EXISTS + lancement du script avec un json et entre 0 et 3 fichiers de métadonnées (personnes, instruments et projets) 3) Dans le script de la base de données : Changement de groupe_recolte en groupe et ajout d'un attribut nom dans groupe et dans projet + ajout DROP TABLE IF EXISTS ... CASCADE pour la table utilisateur
</commit_message>
<xml_diff>
--- a/Base_de_donnees/Fichiers_metadonnees/Metadonnees_instruments_capteurs.xlsx
+++ b/Base_de_donnees/Fichiers_metadonnees/Metadonnees_instruments_capteurs.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Instruments" sheetId="1" state="visible" r:id="rId3"/>
@@ -13,6 +13,7 @@
     <sheet name="Remplace_instrument&amp;capteur" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Coefficients_correcteurs" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Maintenance" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Localisations" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="124">
   <si>
     <t xml:space="preserve">numéro_serie</t>
   </si>
@@ -191,7 +192,7 @@
     <t xml:space="preserve">Dendro_92261195</t>
   </si>
   <si>
-    <t xml:space="preserve">Dendrometre</t>
+    <t xml:space="preserve">Dendromètre</t>
   </si>
   <si>
     <t xml:space="preserve">identifiant_instrument (num_instrument)</t>
@@ -320,9 +321,6 @@
     <t xml:space="preserve">capteur de température du HOBO n°38</t>
   </si>
   <si>
-    <t xml:space="preserve">01/09/2023</t>
-  </si>
-  <si>
     <t xml:space="preserve">capteur de température à -6cm du sol du TMS4 n°0</t>
   </si>
   <si>
@@ -335,9 +333,6 @@
     <t xml:space="preserve">capteur de conductivité du TMS4 n°0</t>
   </si>
   <si>
-    <t xml:space="preserve">01/03/2026</t>
-  </si>
-  <si>
     <t xml:space="preserve">capteur de température du Dendromètre n°0</t>
   </si>
   <si>
@@ -378,18 +373,43 @@
   </si>
   <si>
     <t xml:space="preserve">étalonnage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">altitude</t>
+  </si>
+  <si>
+    <t xml:space="preserve">longitude</t>
+  </si>
+  <si>
+    <t xml:space="preserve">latitude</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hauteur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">orientation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">catégorie_de_milieu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">description_milieu</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yy"/>
+    <numFmt numFmtId="167" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="12">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -440,6 +460,34 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -483,7 +531,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -508,7 +556,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -518,6 +566,26 @@
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -710,7 +778,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I41"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.52"/>
@@ -1594,7 +1662,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E45"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="31.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="25.38"/>
@@ -2148,11 +2216,11 @@
       <c r="A40" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="6" t="n">
+        <v>45170</v>
+      </c>
+      <c r="C40" s="4" t="s">
         <v>98</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>99</v>
       </c>
       <c r="D40" s="1" t="n">
         <v>4</v>
@@ -2162,11 +2230,11 @@
       <c r="A41" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B41" s="6" t="s">
-        <v>98</v>
+      <c r="B41" s="6" t="n">
+        <v>45170</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D41" s="1" t="n">
         <v>5</v>
@@ -2176,53 +2244,53 @@
       <c r="A42" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B42" s="6" t="s">
-        <v>98</v>
+      <c r="B42" s="6" t="n">
+        <v>45170</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D42" s="1" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B43" s="6" t="s">
-        <v>98</v>
+      <c r="B43" s="6" t="n">
+        <v>45170</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D43" s="1" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B44" s="6" t="s">
-        <v>103</v>
+      <c r="B44" s="6" t="n">
+        <v>46082</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D44" s="1" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="6" t="n">
+        <v>46082</v>
+      </c>
+      <c r="C45" s="4" t="s">
         <v>103</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>105</v>
       </c>
       <c r="D45" s="1" t="n">
         <v>7</v>
@@ -2245,7 +2313,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="35.48"/>
@@ -2256,19 +2324,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2292,7 +2360,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C39"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.62"/>
@@ -2302,13 +2370,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2669,7 +2737,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D39"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="34.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="35.75"/>
@@ -2677,16 +2745,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2697,7 +2765,7 @@
         <v>45377</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>60</v>
@@ -2711,7 +2779,7 @@
         <v>45377</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>61</v>
@@ -2725,7 +2793,7 @@
         <v>45377</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>62</v>
@@ -2739,7 +2807,7 @@
         <v>45377</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>63</v>
@@ -2753,7 +2821,7 @@
         <v>45377</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>64</v>
@@ -2767,7 +2835,7 @@
         <v>45377</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>65</v>
@@ -2781,7 +2849,7 @@
         <v>45377</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>66</v>
@@ -2795,7 +2863,7 @@
         <v>45377</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>67</v>
@@ -2809,7 +2877,7 @@
         <v>45377</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>68</v>
@@ -2823,7 +2891,7 @@
         <v>45377</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>69</v>
@@ -2837,7 +2905,7 @@
         <v>45377</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>70</v>
@@ -2851,7 +2919,7 @@
         <v>45377</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>71</v>
@@ -2865,7 +2933,7 @@
         <v>45377</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>72</v>
@@ -2879,7 +2947,7 @@
         <v>45377</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>73</v>
@@ -2893,7 +2961,7 @@
         <v>45377</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>74</v>
@@ -2907,7 +2975,7 @@
         <v>45377</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>75</v>
@@ -2921,7 +2989,7 @@
         <v>45377</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>76</v>
@@ -2935,7 +3003,7 @@
         <v>45377</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>77</v>
@@ -2949,7 +3017,7 @@
         <v>45377</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>78</v>
@@ -2963,7 +3031,7 @@
         <v>45377</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>79</v>
@@ -2977,7 +3045,7 @@
         <v>45377</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>80</v>
@@ -2991,7 +3059,7 @@
         <v>45377</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>81</v>
@@ -3005,7 +3073,7 @@
         <v>45377</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>82</v>
@@ -3019,7 +3087,7 @@
         <v>45377</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>83</v>
@@ -3033,7 +3101,7 @@
         <v>45377</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>84</v>
@@ -3047,7 +3115,7 @@
         <v>45377</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>85</v>
@@ -3061,7 +3129,7 @@
         <v>45377</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>86</v>
@@ -3075,7 +3143,7 @@
         <v>45377</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>87</v>
@@ -3089,7 +3157,7 @@
         <v>45377</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>88</v>
@@ -3103,7 +3171,7 @@
         <v>45377</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>89</v>
@@ -3117,7 +3185,7 @@
         <v>45377</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>90</v>
@@ -3131,7 +3199,7 @@
         <v>45377</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>91</v>
@@ -3145,7 +3213,7 @@
         <v>45377</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>92</v>
@@ -3159,7 +3227,7 @@
         <v>45377</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>93</v>
@@ -3173,7 +3241,7 @@
         <v>45377</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D36" s="4" t="s">
         <v>94</v>
@@ -3187,7 +3255,7 @@
         <v>45377</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>95</v>
@@ -3201,7 +3269,7 @@
         <v>45377</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>96</v>
@@ -3215,7 +3283,7 @@
         <v>45377</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>97</v>
@@ -3230,4 +3298,587 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:K41"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="38.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="3" style="1" width="12.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="21.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="33.94"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>45412</v>
+      </c>
+      <c r="C2" s="4"/>
+      <c r="E2" s="10" t="n">
+        <v>3.861986</v>
+      </c>
+      <c r="F2" s="10" t="n">
+        <v>43.6321572</v>
+      </c>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+    </row>
+    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>45412</v>
+      </c>
+      <c r="C3" s="4"/>
+      <c r="E3" s="10" t="n">
+        <v>3.8622103</v>
+      </c>
+      <c r="F3" s="10" t="n">
+        <v>43.6317276</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>45412</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="E4" s="10" t="n">
+        <v>3.8627119</v>
+      </c>
+      <c r="F4" s="10" t="n">
+        <v>43.6322906</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>45412</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>3.8633402</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>43.6325401</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>45412</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>3.8614151</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>43.6319594</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>45412</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>3.8613255</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>43.6317551</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>45412</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>3.8616474</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>43.6319312</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>45412</v>
+      </c>
+      <c r="E9" s="10" t="n">
+        <v>3.8620541</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>43.6316813</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>45412</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>3.863478</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>43.6312265</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>45412</v>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>3.8641962</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>43.6311804</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>45412</v>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>3.8646169</v>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>43.6311144</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>45412</v>
+      </c>
+      <c r="E13" s="10" t="n">
+        <v>3.8651054</v>
+      </c>
+      <c r="F13" s="10" t="n">
+        <v>43.6310513</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>45412</v>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>3.8659849</v>
+      </c>
+      <c r="F14" s="10" t="n">
+        <v>43.6307912</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>45412</v>
+      </c>
+      <c r="E15" s="10" t="n">
+        <v>3.8646428</v>
+      </c>
+      <c r="F15" s="10" t="n">
+        <v>43.6331516</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>45412</v>
+      </c>
+      <c r="E16" s="10" t="n">
+        <v>3.8651061</v>
+      </c>
+      <c r="F16" s="10" t="n">
+        <v>43.6332261</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>45412</v>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>3.8652986</v>
+      </c>
+      <c r="F17" s="10" t="n">
+        <v>43.633271</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>45412</v>
+      </c>
+      <c r="E18" s="10" t="n">
+        <v>3.8655825</v>
+      </c>
+      <c r="F18" s="10" t="n">
+        <v>43.6334355</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>45451</v>
+      </c>
+      <c r="E19" s="11" t="n">
+        <v>3.8611136</v>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>43.6321676</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>45451</v>
+      </c>
+      <c r="E20" s="11" t="n">
+        <v>3.8627079</v>
+      </c>
+      <c r="F20" s="11" t="n">
+        <v>43.6320455</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>45451</v>
+      </c>
+      <c r="E21" s="11" t="n">
+        <v>3.8640141</v>
+      </c>
+      <c r="F21" s="11" t="n">
+        <v>43.6322195</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>45451</v>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v>3.8635337</v>
+      </c>
+      <c r="F22" s="11" t="n">
+        <v>43.63242</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>45451</v>
+      </c>
+      <c r="E23" s="11" t="n">
+        <v>3.8655151</v>
+      </c>
+      <c r="F23" s="11" t="n">
+        <v>43.6332739</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>45451</v>
+      </c>
+      <c r="E24" s="11" t="n">
+        <v>3.8631799</v>
+      </c>
+      <c r="F24" s="11" t="n">
+        <v>43.6327381</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>45451</v>
+      </c>
+      <c r="E25" s="11" t="n">
+        <v>3.8620876</v>
+      </c>
+      <c r="F25" s="11" t="n">
+        <v>43.6339619</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>45451</v>
+      </c>
+      <c r="E26" s="11" t="n">
+        <v>3.8650515</v>
+      </c>
+      <c r="F26" s="11" t="n">
+        <v>43.6331601</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>45451</v>
+      </c>
+      <c r="E27" s="11" t="n">
+        <v>3.8621486</v>
+      </c>
+      <c r="F27" s="11" t="n">
+        <v>43.6341674</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>45451</v>
+      </c>
+      <c r="E28" s="11" t="n">
+        <v>3.8626422</v>
+      </c>
+      <c r="F28" s="11" t="n">
+        <v>43.6324899</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>45451</v>
+      </c>
+      <c r="E29" s="11" t="n">
+        <v>3.8623371</v>
+      </c>
+      <c r="F29" s="11" t="n">
+        <v>43.6337978</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B30" s="5"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+    </row>
+    <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>45451</v>
+      </c>
+      <c r="E31" s="11" t="n">
+        <v>3.8660932</v>
+      </c>
+      <c r="F31" s="11" t="n">
+        <v>43.6307572</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>45451</v>
+      </c>
+      <c r="E32" s="11" t="n">
+        <v>3.8649371</v>
+      </c>
+      <c r="F32" s="11" t="n">
+        <v>43.6312202</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="5"/>
+      <c r="E33" s="12"/>
+      <c r="F33" s="12"/>
+    </row>
+    <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>45451</v>
+      </c>
+      <c r="E34" s="11" t="n">
+        <v>3.8623052</v>
+      </c>
+      <c r="F34" s="11" t="n">
+        <v>43.633519</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B35" s="5"/>
+      <c r="E35" s="12"/>
+      <c r="F35" s="12"/>
+    </row>
+    <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B36" s="5"/>
+      <c r="E36" s="12"/>
+      <c r="F36" s="12"/>
+    </row>
+    <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>45451</v>
+      </c>
+      <c r="E37" s="11" t="n">
+        <v>3.863817</v>
+      </c>
+      <c r="F37" s="11" t="n">
+        <v>43.6311266</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B38" s="5"/>
+      <c r="E38" s="12"/>
+      <c r="F38" s="12"/>
+    </row>
+    <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>45451</v>
+      </c>
+      <c r="E39" s="11" t="n">
+        <v>3.861869</v>
+      </c>
+      <c r="F39" s="11" t="n">
+        <v>43.6321227</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>45170</v>
+      </c>
+      <c r="E40" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B41" s="13" t="n">
+        <v>46082</v>
+      </c>
+      <c r="E41" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Script d'intégration des metadonnées et JSON : - exemple de JSON pour l'intégration de metadonnées : integration_meta.json - Prise en compte du fait que si les cases des excels contenant des informations nécessaires sont vides alors violation des contraintes NOT NULL. Solution : ajout de WHERE ... IS NOT NULL dans les INSERT et des tests de remplissage des cases des excels (if row[n] != None : ...)
</commit_message>
<xml_diff>
--- a/Base_de_donnees/Fichiers_metadonnees/Metadonnees_instruments_capteurs.xlsx
+++ b/Base_de_donnees/Fichiers_metadonnees/Metadonnees_instruments_capteurs.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="166">
   <si>
     <t xml:space="preserve">numéro_serie</t>
   </si>
@@ -201,148 +201,280 @@
     <t xml:space="preserve">date_activation (YYYY/MM/DD)</t>
   </si>
   <si>
-    <t xml:space="preserve">description (unique)</t>
-  </si>
-  <si>
     <t xml:space="preserve">num_colonne</t>
   </si>
   <si>
+    <t xml:space="preserve">nom_capteur</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°01</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°01_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°02</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°02_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°03</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°03_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°04</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°04_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°05</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°05_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°06</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°06_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°07</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°07_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°08</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°08_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°09</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°09_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°10</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°10_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°11</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°11_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°12</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°12_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°13</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°13_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°14</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°14_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°15</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°15_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°16</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°16_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°17</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°17_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°18</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°18_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°19</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°19_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°20</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°20_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°21</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°21_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°22</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°22_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°23</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°23_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°24</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°24_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°25</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°25_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°26</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°26_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°27</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°27_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°28</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°28_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°29</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°29_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°30</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°30_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°31</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°31_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°32</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°32_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°33</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°33_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°34</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°34_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°35</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°35_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°36</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°36_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°37</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°37_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du HOBO n°38</t>
   </si>
   <si>
+    <t xml:space="preserve">HOBO_n°38_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température à -6cm du sol du TMS4 n°0</t>
   </si>
   <si>
+    <t xml:space="preserve">TMS4_95224601_temp_-6</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température à 2cm du sol du TMS4 n°0</t>
   </si>
   <si>
+    <t xml:space="preserve">TMS4_95224601_temp_2</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température à 15cm du sol du TMS4 n°0</t>
   </si>
   <si>
+    <t xml:space="preserve">TMS4_95224601_temp_15</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de conductivité du TMS4 n°0</t>
   </si>
   <si>
+    <t xml:space="preserve">TMS4_95224601_cond</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de température du Dendromètre n°0</t>
   </si>
   <si>
+    <t xml:space="preserve">Dendro_92261195_temp</t>
+  </si>
+  <si>
     <t xml:space="preserve">capteur de variation de diamètre du Dendromètre n°0</t>
   </si>
   <si>
-    <t xml:space="preserve">id_initial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id_nouveau</t>
+    <t xml:space="preserve">Dendro_92261195_diam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">num_instr/nom_capt_à_remplacer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">num_instr/nom_capt_remplaçant</t>
   </si>
   <si>
     <t xml:space="preserve">date_remplacement (YYYY/MM/DD)</t>
@@ -360,16 +492,10 @@
     <t xml:space="preserve">date_calibration</t>
   </si>
   <si>
-    <t xml:space="preserve">description_capteur</t>
-  </si>
-  <si>
     <t xml:space="preserve">date_debut</t>
   </si>
   <si>
     <t xml:space="preserve">date_fin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">description capteur</t>
   </si>
   <si>
     <t xml:space="preserve">étalonnage</t>
@@ -409,7 +535,7 @@
     <numFmt numFmtId="166" formatCode="dd/mm/yy"/>
     <numFmt numFmtId="167" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -459,6 +585,18 @@
       <name val="Aptos"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="0"/>
     </font>
     <font>
       <sz val="11"/>
@@ -531,7 +669,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -560,11 +698,7 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -576,6 +710,14 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -584,8 +726,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1661,7 +1807,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="31.88"/>
@@ -1679,12 +1825,14 @@
         <v>57</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="E1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
@@ -1699,6 +1847,9 @@
       <c r="D2" s="1" t="n">
         <v>3</v>
       </c>
+      <c r="E2" s="1" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
@@ -1708,10 +1859,13 @@
         <v>45412</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D3" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1722,10 +1876,13 @@
         <v>45412</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1736,10 +1893,13 @@
         <v>45412</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D5" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1750,10 +1910,13 @@
         <v>45412</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1764,10 +1927,13 @@
         <v>45412</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D7" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1778,10 +1944,13 @@
         <v>45412</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D8" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1792,10 +1961,13 @@
         <v>45412</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1806,10 +1978,13 @@
         <v>45412</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="D10" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1820,10 +1995,13 @@
         <v>45412</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="D11" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1834,10 +2012,13 @@
         <v>45412</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="D12" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1848,10 +2029,13 @@
         <v>45412</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="D13" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1862,10 +2046,13 @@
         <v>45412</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="D14" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1876,10 +2063,13 @@
         <v>45412</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="D15" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1890,10 +2080,13 @@
         <v>45412</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="D16" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1904,10 +2097,13 @@
         <v>45412</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="D17" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1918,10 +2114,13 @@
         <v>45412</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="D18" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1932,10 +2131,13 @@
         <v>45451</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="D19" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1946,10 +2148,13 @@
         <v>45451</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="D20" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1960,10 +2165,13 @@
         <v>45451</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="D21" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1974,10 +2182,13 @@
         <v>45451</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="D22" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1988,10 +2199,13 @@
         <v>45451</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="D23" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2002,10 +2216,13 @@
         <v>45451</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>82</v>
+        <v>104</v>
       </c>
       <c r="D24" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2016,10 +2233,13 @@
         <v>45451</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="D25" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2030,10 +2250,13 @@
         <v>45451</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="D26" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2044,10 +2267,13 @@
         <v>45451</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>85</v>
+        <v>110</v>
       </c>
       <c r="D27" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2058,10 +2284,13 @@
         <v>45451</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>86</v>
+        <v>112</v>
       </c>
       <c r="D28" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2072,10 +2301,13 @@
         <v>45451</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>87</v>
+        <v>114</v>
       </c>
       <c r="D29" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2086,10 +2318,13 @@
         <v>46098</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>88</v>
+        <v>116</v>
       </c>
       <c r="D30" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2100,10 +2335,13 @@
         <v>45451</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>89</v>
+        <v>118</v>
       </c>
       <c r="D31" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2114,10 +2352,13 @@
         <v>45451</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="D32" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2128,10 +2369,13 @@
         <v>46098</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>91</v>
+        <v>122</v>
       </c>
       <c r="D33" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2142,10 +2386,13 @@
         <v>45451</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>92</v>
+        <v>124</v>
       </c>
       <c r="D34" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2154,10 +2401,13 @@
       </c>
       <c r="B35" s="5"/>
       <c r="C35" s="4" t="s">
-        <v>93</v>
+        <v>126</v>
       </c>
       <c r="D35" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2166,10 +2416,13 @@
       </c>
       <c r="B36" s="5"/>
       <c r="C36" s="4" t="s">
-        <v>94</v>
+        <v>128</v>
       </c>
       <c r="D36" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2180,10 +2433,13 @@
         <v>45451</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>95</v>
+        <v>130</v>
       </c>
       <c r="D37" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2192,10 +2448,13 @@
       </c>
       <c r="B38" s="5"/>
       <c r="C38" s="4" t="s">
-        <v>96</v>
+        <v>132</v>
       </c>
       <c r="D38" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2206,10 +2465,13 @@
         <v>45451</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>97</v>
+        <v>134</v>
       </c>
       <c r="D39" s="1" t="n">
         <v>3</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2220,10 +2482,13 @@
         <v>45170</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>98</v>
+        <v>136</v>
       </c>
       <c r="D40" s="1" t="n">
         <v>4</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2234,10 +2499,13 @@
         <v>45170</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>99</v>
+        <v>138</v>
       </c>
       <c r="D41" s="1" t="n">
         <v>5</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2248,10 +2516,13 @@
         <v>45170</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>100</v>
+        <v>140</v>
       </c>
       <c r="D42" s="1" t="n">
         <v>6</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2262,10 +2533,13 @@
         <v>45170</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>101</v>
+        <v>142</v>
       </c>
       <c r="D43" s="1" t="n">
         <v>7</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2276,10 +2550,13 @@
         <v>46082</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>102</v>
+        <v>144</v>
       </c>
       <c r="D44" s="1" t="n">
         <v>4</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2290,11 +2567,18 @@
         <v>46082</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>103</v>
+        <v>146</v>
       </c>
       <c r="D45" s="1" t="n">
         <v>7</v>
       </c>
+      <c r="E45" s="1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B47" s="7"/>
+      <c r="E47" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2315,33 +2599,34 @@
   <dimension ref="A1:E3"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="35.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="27.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="43.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="38.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="34.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="24.21"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="20.25"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>105</v>
+        <v>148</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>149</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>106</v>
+        <v>150</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>107</v>
+        <v>151</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>108</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="7"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2364,361 +2649,350 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="32.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="25.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="21.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>109</v>
+        <v>153</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>110</v>
+        <v>154</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>111</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="n">
         <v>-0.09653415444</v>
       </c>
-      <c r="B2" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>61</v>
+      <c r="B2" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <v>-0.08044650796</v>
       </c>
-      <c r="B3" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>62</v>
+      <c r="B3" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="n">
         <v>0.05317033367</v>
       </c>
-      <c r="B4" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>63</v>
+      <c r="B4" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="n">
         <v>-0.0570970766</v>
       </c>
-      <c r="B5" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>64</v>
+      <c r="B5" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
         <v>-0.05486268126</v>
       </c>
-      <c r="B6" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>65</v>
+      <c r="B6" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="n">
         <v>-0.03564688129</v>
       </c>
-      <c r="B7" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>66</v>
+      <c r="B7" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
         <v>-0.1518354392</v>
       </c>
-      <c r="B8" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>68</v>
+      <c r="B8" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="n">
         <v>-0.07340816262</v>
       </c>
-      <c r="B9" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>70</v>
+      <c r="B9" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="n">
         <v>-0.06167758706</v>
       </c>
-      <c r="B10" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>71</v>
+      <c r="B10" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="n">
         <v>0.005689432592</v>
       </c>
-      <c r="B11" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>72</v>
+      <c r="B11" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="n">
         <v>0.06635326621</v>
       </c>
-      <c r="B12" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>73</v>
+      <c r="B12" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="n">
         <v>0.06724702435</v>
       </c>
-      <c r="B13" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>74</v>
+      <c r="B13" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="n">
         <v>0.1786316323</v>
       </c>
-      <c r="B14" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>75</v>
+      <c r="B14" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="n">
         <v>0.0766314848</v>
       </c>
-      <c r="B15" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>76</v>
+      <c r="B15" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="n">
         <v>0.1915911253</v>
       </c>
-      <c r="B16" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>77</v>
+      <c r="B16" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="n">
         <v>0.1263467812</v>
       </c>
-      <c r="B17" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>78</v>
+      <c r="B17" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="n">
         <v>0.1069075417</v>
       </c>
-      <c r="B18" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>79</v>
+      <c r="B18" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="n">
         <v>0.1437750649</v>
       </c>
-      <c r="B19" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>80</v>
+      <c r="B19" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="n">
         <v>-0.02615070108</v>
       </c>
-      <c r="B20" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>81</v>
+      <c r="B20" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="n">
         <v>0.1119349312</v>
       </c>
-      <c r="B21" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>82</v>
+      <c r="B21" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="n">
         <v>-0.1126218009</v>
       </c>
-      <c r="B22" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>83</v>
+      <c r="B22" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="n">
         <v>-0.09698103351</v>
       </c>
-      <c r="B23" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>84</v>
+      <c r="B23" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="n">
         <v>0.006136311661</v>
       </c>
-      <c r="B24" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>85</v>
+      <c r="B24" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="n">
         <v>-0.02324598713</v>
       </c>
-      <c r="B25" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>87</v>
+      <c r="B25" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="n">
         <v>-0.05519784056</v>
       </c>
-      <c r="B26" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>89</v>
+      <c r="B26" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="n">
         <v>-0.0697214103</v>
       </c>
-      <c r="B27" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>90</v>
+      <c r="B27" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="n">
         <v>-0.138987666</v>
       </c>
-      <c r="B28" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>95</v>
+      <c r="B28" s="10" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="7"/>
-      <c r="C29" s="4"/>
+      <c r="B29" s="10"/>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="7"/>
-      <c r="C30" s="4"/>
+      <c r="B30" s="10"/>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="7"/>
-      <c r="C31" s="4"/>
+      <c r="B31" s="10"/>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="7"/>
-      <c r="C32" s="4"/>
+      <c r="B32" s="10"/>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="7"/>
-      <c r="C33" s="4"/>
+      <c r="B33" s="10"/>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="7"/>
-      <c r="C34" s="4"/>
+      <c r="B34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="7"/>
-      <c r="C35" s="4"/>
+      <c r="B35" s="10"/>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="7"/>
-      <c r="C36" s="4"/>
+      <c r="B36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="7"/>
-      <c r="C37" s="4"/>
+      <c r="B37" s="10"/>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="7"/>
-      <c r="C38" s="4"/>
+      <c r="B38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B39" s="7"/>
-      <c r="C39" s="4"/>
+      <c r="B39" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2740,553 +3014,554 @@
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="34.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="35.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="21.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>112</v>
+        <v>155</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>113</v>
+        <v>156</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>114</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="n">
+      <c r="A2" s="10" t="n">
         <v>45372</v>
       </c>
-      <c r="B2" s="8" t="n">
+      <c r="B2" s="11" t="n">
         <v>45377</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B3" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B11" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B13" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B14" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B16" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B17" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B18" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B19" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B20" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B21" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B22" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B23" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B24" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B25" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B26" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B27" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B28" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B29" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D29" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="n">
+    </row>
+    <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="10" t="n">
         <v>45372</v>
       </c>
-      <c r="B3" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="n">
+      <c r="B30" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="10" t="n">
         <v>45372</v>
       </c>
-      <c r="B4" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="n">
+      <c r="B31" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="10" t="n">
         <v>45372</v>
       </c>
-      <c r="B5" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="n">
+      <c r="B32" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="10" t="n">
         <v>45372</v>
       </c>
-      <c r="B6" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="n">
+      <c r="B33" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="10" t="n">
         <v>45372</v>
       </c>
-      <c r="B7" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="n">
+      <c r="B34" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="10" t="n">
         <v>45372</v>
       </c>
-      <c r="B8" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="n">
+      <c r="B35" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="10" t="n">
         <v>45372</v>
       </c>
-      <c r="B9" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="n">
+      <c r="B36" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="10" t="n">
         <v>45372</v>
       </c>
-      <c r="B10" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="n">
+      <c r="B37" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="10" t="n">
         <v>45372</v>
       </c>
-      <c r="B11" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="n">
+      <c r="B38" s="11" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="10" t="n">
         <v>45372</v>
       </c>
-      <c r="B12" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B13" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B14" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B15" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B16" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B17" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B18" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B19" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B20" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B21" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B22" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B23" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B24" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B25" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B26" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B27" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B28" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B29" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B30" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B31" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B32" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B33" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B34" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B35" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B36" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D36" s="4" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B37" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B38" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B39" s="8" t="n">
+      <c r="B39" s="11" t="n">
         <v>45377</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>97</v>
+        <v>157</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -3320,34 +3595,34 @@
         <v>56</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>112</v>
+        <v>155</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>113</v>
+        <v>156</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>116</v>
+        <v>158</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>117</v>
+        <v>159</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>118</v>
+        <v>160</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>119</v>
+        <v>161</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>120</v>
+        <v>162</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="J1" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="K1" s="9" t="s">
-        <v>123</v>
+        <v>163</v>
+      </c>
+      <c r="J1" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="K1" s="12" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3358,10 +3633,10 @@
         <v>45412</v>
       </c>
       <c r="C2" s="4"/>
-      <c r="E2" s="10" t="n">
+      <c r="E2" s="13" t="n">
         <v>3.861986</v>
       </c>
-      <c r="F2" s="10" t="n">
+      <c r="F2" s="13" t="n">
         <v>43.6321572</v>
       </c>
       <c r="G2" s="4"/>
@@ -3377,10 +3652,10 @@
         <v>45412</v>
       </c>
       <c r="C3" s="4"/>
-      <c r="E3" s="10" t="n">
+      <c r="E3" s="13" t="n">
         <v>3.8622103</v>
       </c>
-      <c r="F3" s="10" t="n">
+      <c r="F3" s="13" t="n">
         <v>43.6317276</v>
       </c>
     </row>
@@ -3392,10 +3667,10 @@
         <v>45412</v>
       </c>
       <c r="C4" s="4"/>
-      <c r="E4" s="10" t="n">
+      <c r="E4" s="13" t="n">
         <v>3.8627119</v>
       </c>
-      <c r="F4" s="10" t="n">
+      <c r="F4" s="13" t="n">
         <v>43.6322906</v>
       </c>
     </row>
@@ -3406,10 +3681,10 @@
       <c r="B5" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="E5" s="13" t="n">
         <v>3.8633402</v>
       </c>
-      <c r="F5" s="10" t="n">
+      <c r="F5" s="13" t="n">
         <v>43.6325401</v>
       </c>
     </row>
@@ -3420,10 +3695,10 @@
       <c r="B6" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="E6" s="10" t="n">
+      <c r="E6" s="13" t="n">
         <v>3.8614151</v>
       </c>
-      <c r="F6" s="10" t="n">
+      <c r="F6" s="13" t="n">
         <v>43.6319594</v>
       </c>
     </row>
@@ -3434,10 +3709,10 @@
       <c r="B7" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="E7" s="13" t="n">
         <v>3.8613255</v>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="F7" s="13" t="n">
         <v>43.6317551</v>
       </c>
     </row>
@@ -3448,10 +3723,10 @@
       <c r="B8" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="E8" s="10" t="n">
+      <c r="E8" s="13" t="n">
         <v>3.8616474</v>
       </c>
-      <c r="F8" s="10" t="n">
+      <c r="F8" s="13" t="n">
         <v>43.6319312</v>
       </c>
     </row>
@@ -3462,10 +3737,10 @@
       <c r="B9" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="13" t="n">
         <v>3.8620541</v>
       </c>
-      <c r="F9" s="10" t="n">
+      <c r="F9" s="13" t="n">
         <v>43.6316813</v>
       </c>
     </row>
@@ -3476,10 +3751,10 @@
       <c r="B10" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="E10" s="10" t="n">
+      <c r="E10" s="13" t="n">
         <v>3.863478</v>
       </c>
-      <c r="F10" s="10" t="n">
+      <c r="F10" s="13" t="n">
         <v>43.6312265</v>
       </c>
     </row>
@@ -3490,10 +3765,10 @@
       <c r="B11" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E11" s="13" t="n">
         <v>3.8641962</v>
       </c>
-      <c r="F11" s="10" t="n">
+      <c r="F11" s="13" t="n">
         <v>43.6311804</v>
       </c>
     </row>
@@ -3504,10 +3779,10 @@
       <c r="B12" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="E12" s="10" t="n">
+      <c r="E12" s="13" t="n">
         <v>3.8646169</v>
       </c>
-      <c r="F12" s="10" t="n">
+      <c r="F12" s="13" t="n">
         <v>43.6311144</v>
       </c>
     </row>
@@ -3518,10 +3793,10 @@
       <c r="B13" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E13" s="13" t="n">
         <v>3.8651054</v>
       </c>
-      <c r="F13" s="10" t="n">
+      <c r="F13" s="13" t="n">
         <v>43.6310513</v>
       </c>
     </row>
@@ -3532,10 +3807,10 @@
       <c r="B14" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="E14" s="10" t="n">
+      <c r="E14" s="13" t="n">
         <v>3.8659849</v>
       </c>
-      <c r="F14" s="10" t="n">
+      <c r="F14" s="13" t="n">
         <v>43.6307912</v>
       </c>
     </row>
@@ -3546,10 +3821,10 @@
       <c r="B15" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="E15" s="10" t="n">
+      <c r="E15" s="13" t="n">
         <v>3.8646428</v>
       </c>
-      <c r="F15" s="10" t="n">
+      <c r="F15" s="13" t="n">
         <v>43.6331516</v>
       </c>
     </row>
@@ -3560,10 +3835,10 @@
       <c r="B16" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="E16" s="13" t="n">
         <v>3.8651061</v>
       </c>
-      <c r="F16" s="10" t="n">
+      <c r="F16" s="13" t="n">
         <v>43.6332261</v>
       </c>
     </row>
@@ -3574,10 +3849,10 @@
       <c r="B17" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="E17" s="10" t="n">
+      <c r="E17" s="13" t="n">
         <v>3.8652986</v>
       </c>
-      <c r="F17" s="10" t="n">
+      <c r="F17" s="13" t="n">
         <v>43.633271</v>
       </c>
     </row>
@@ -3588,10 +3863,10 @@
       <c r="B18" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="E18" s="10" t="n">
+      <c r="E18" s="13" t="n">
         <v>3.8655825</v>
       </c>
-      <c r="F18" s="10" t="n">
+      <c r="F18" s="13" t="n">
         <v>43.6334355</v>
       </c>
     </row>
@@ -3602,10 +3877,10 @@
       <c r="B19" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="E19" s="11" t="n">
+      <c r="E19" s="14" t="n">
         <v>3.8611136</v>
       </c>
-      <c r="F19" s="11" t="n">
+      <c r="F19" s="14" t="n">
         <v>43.6321676</v>
       </c>
     </row>
@@ -3616,10 +3891,10 @@
       <c r="B20" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="E20" s="11" t="n">
+      <c r="E20" s="14" t="n">
         <v>3.8627079</v>
       </c>
-      <c r="F20" s="11" t="n">
+      <c r="F20" s="14" t="n">
         <v>43.6320455</v>
       </c>
     </row>
@@ -3630,10 +3905,10 @@
       <c r="B21" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="E21" s="11" t="n">
+      <c r="E21" s="14" t="n">
         <v>3.8640141</v>
       </c>
-      <c r="F21" s="11" t="n">
+      <c r="F21" s="14" t="n">
         <v>43.6322195</v>
       </c>
     </row>
@@ -3644,10 +3919,10 @@
       <c r="B22" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="E22" s="11" t="n">
+      <c r="E22" s="14" t="n">
         <v>3.8635337</v>
       </c>
-      <c r="F22" s="11" t="n">
+      <c r="F22" s="14" t="n">
         <v>43.63242</v>
       </c>
     </row>
@@ -3658,10 +3933,10 @@
       <c r="B23" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="E23" s="11" t="n">
+      <c r="E23" s="14" t="n">
         <v>3.8655151</v>
       </c>
-      <c r="F23" s="11" t="n">
+      <c r="F23" s="14" t="n">
         <v>43.6332739</v>
       </c>
     </row>
@@ -3672,10 +3947,10 @@
       <c r="B24" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="E24" s="11" t="n">
+      <c r="E24" s="14" t="n">
         <v>3.8631799</v>
       </c>
-      <c r="F24" s="11" t="n">
+      <c r="F24" s="14" t="n">
         <v>43.6327381</v>
       </c>
     </row>
@@ -3686,10 +3961,10 @@
       <c r="B25" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="E25" s="11" t="n">
+      <c r="E25" s="14" t="n">
         <v>3.8620876</v>
       </c>
-      <c r="F25" s="11" t="n">
+      <c r="F25" s="14" t="n">
         <v>43.6339619</v>
       </c>
     </row>
@@ -3700,10 +3975,10 @@
       <c r="B26" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="E26" s="11" t="n">
+      <c r="E26" s="14" t="n">
         <v>3.8650515</v>
       </c>
-      <c r="F26" s="11" t="n">
+      <c r="F26" s="14" t="n">
         <v>43.6331601</v>
       </c>
     </row>
@@ -3714,10 +3989,10 @@
       <c r="B27" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="E27" s="11" t="n">
+      <c r="E27" s="14" t="n">
         <v>3.8621486</v>
       </c>
-      <c r="F27" s="11" t="n">
+      <c r="F27" s="14" t="n">
         <v>43.6341674</v>
       </c>
     </row>
@@ -3728,10 +4003,10 @@
       <c r="B28" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="E28" s="11" t="n">
+      <c r="E28" s="14" t="n">
         <v>3.8626422</v>
       </c>
-      <c r="F28" s="11" t="n">
+      <c r="F28" s="14" t="n">
         <v>43.6324899</v>
       </c>
     </row>
@@ -3742,17 +4017,17 @@
       <c r="B29" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="E29" s="11" t="n">
+      <c r="E29" s="14" t="n">
         <v>3.8623371</v>
       </c>
-      <c r="F29" s="11" t="n">
+      <c r="F29" s="14" t="n">
         <v>43.6337978</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="5"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="12"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
@@ -3761,10 +4036,10 @@
       <c r="B31" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="E31" s="11" t="n">
+      <c r="E31" s="14" t="n">
         <v>3.8660932</v>
       </c>
-      <c r="F31" s="11" t="n">
+      <c r="F31" s="14" t="n">
         <v>43.6307572</v>
       </c>
     </row>
@@ -3775,17 +4050,17 @@
       <c r="B32" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="E32" s="11" t="n">
+      <c r="E32" s="14" t="n">
         <v>3.8649371</v>
       </c>
-      <c r="F32" s="11" t="n">
+      <c r="F32" s="14" t="n">
         <v>43.6312202</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="5"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="12"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
@@ -3794,22 +4069,22 @@
       <c r="B34" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="E34" s="11" t="n">
+      <c r="E34" s="14" t="n">
         <v>3.8623052</v>
       </c>
-      <c r="F34" s="11" t="n">
+      <c r="F34" s="14" t="n">
         <v>43.633519</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="5"/>
-      <c r="E35" s="12"/>
-      <c r="F35" s="12"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="5"/>
-      <c r="E36" s="12"/>
-      <c r="F36" s="12"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
@@ -3818,17 +4093,17 @@
       <c r="B37" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="E37" s="11" t="n">
+      <c r="E37" s="14" t="n">
         <v>3.863817</v>
       </c>
-      <c r="F37" s="11" t="n">
+      <c r="F37" s="14" t="n">
         <v>43.6311266</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="5"/>
-      <c r="E38" s="12"/>
-      <c r="F38" s="12"/>
+      <c r="E38" s="15"/>
+      <c r="F38" s="15"/>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
@@ -3837,10 +4112,10 @@
       <c r="B39" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="E39" s="11" t="n">
+      <c r="E39" s="14" t="n">
         <v>3.861869</v>
       </c>
-      <c r="F39" s="11" t="n">
+      <c r="F39" s="14" t="n">
         <v>43.6321227</v>
       </c>
     </row>
@@ -3862,7 +4137,7 @@
       <c r="A41" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B41" s="13" t="n">
+      <c r="B41" s="6" t="n">
         <v>46082</v>
       </c>
       <c r="E41" s="1" t="n">

</xml_diff>